<commit_message>
Batch Multi-Format Conversion: text-content.xlsx
</commit_message>
<xml_diff>
--- a/text-content.xlsx
+++ b/text-content.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -447,6 +447,7 @@
           <t>Status</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -479,6 +480,7 @@
           <t>In Progress</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -511,6 +513,7 @@
           <t>Backlog</t>
         </is>
       </c>
+      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -540,9 +543,23 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
+          <t>Pending"""</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    output_filename="test-strategy</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Universal Multi-Format Deployment: text-content.xlsx
</commit_message>
<xml_diff>
--- a/text-content.xlsx
+++ b/text-content.xlsx
@@ -462,78 +462,1683 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:K32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="50" customWidth="1" min="10" max="10"/>
+    <col width="50" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>Module</t>
+          <t>Scenario ID</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>User Story ID</t>
+          <t>Scenario Title</t>
         </is>
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>Title</t>
+          <t>Test Case ID</t>
         </is>
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <t>Priority</t>
+          <t>Test Case Title</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Preconditions</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Test Type</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Automation Feasible</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Step #</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Test Step Description</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>TC001</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>US-001</t>
+          <t>US32275</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Login Page</t>
+          <t>Plan Recommendation</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Verify side-by-side plan comparison</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>User is logged into the CareSource enrollment portal and has completed the health needs questionnaire</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>User with completed profile and at least two recommended plans</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>Navigate to plan recommendation page</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="inlineStr">
+        <is>
+          <t>System displays side-by-side comparison of at least two plans highlighting premiums, deductibles, co-pays, out-of-pocket maximums, and coverage for specified medications and doctors</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Dashboard</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>US-002</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>User Stats</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Medium</t>
+      <c r="A3" s="3" t="inlineStr"/>
+      <c r="B3" s="3" t="inlineStr"/>
+      <c r="C3" s="3" t="inlineStr"/>
+      <c r="D3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="inlineStr"/>
+      <c r="F3" s="3" t="inlineStr"/>
+      <c r="G3" s="3" t="inlineStr"/>
+      <c r="H3" s="3" t="inlineStr"/>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>Review plan features and select a plan</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>Selected plan is highlighted and user can proceed to enrollment</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>TC002</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>US32275</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Plan Recommendation</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Verify navigation to enrollment after plan selection</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>User is on the plan comparison page</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>User with at least one recommended plan</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Select a plan and click 'Enroll'</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>System transitions to the enrollment process with the chosen plan pre-selected</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>TC003</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>US32275</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Plan Recommendation</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Negative - No recommended plans</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>User has completed health needs but no plans match criteria</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>User with uncommon criteria resulting in no matches</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>Navigate to plan recommendation page</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>System displays a message: "No plans match your criteria. Please adjust your preferences."</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>TC004</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>US32275</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Plan Recommendation</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Edge - Maximum number of plans</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>User qualifies for 10+ plans</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>User with broad criteria resulting in maximum recommendations</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>Navigate to plan recommendation page</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>System displays all recommended plans in a scrollable, readable format without UI breakage</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>TC005</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>US32274</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Plan Personalization</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Verify member can input medications and providers</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>User is authenticated</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Medication: Metformin 500mg, Provider: Dr. Smith</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>Navigate to health needs input page</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>System displays input fields for medications and providers</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr"/>
+      <c r="B8" s="3" t="inlineStr"/>
+      <c r="C8" s="3" t="inlineStr"/>
+      <c r="D8" s="3" t="inlineStr"/>
+      <c r="E8" s="3" t="inlineStr"/>
+      <c r="F8" s="3" t="inlineStr"/>
+      <c r="G8" s="3" t="inlineStr"/>
+      <c r="H8" s="3" t="inlineStr"/>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>Enter medication and provider information and submit</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>System accepts input, validates data, and confirms successful entry</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>TC006</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>US32274</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Plan Personalization</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Verify financial preference input</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>User is authenticated</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>Premium: $200, Deductible: $1000, OOP Max: $5000</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>Navigate to financial preferences section</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>System displays fields for premium, deductible, and out-of-pocket maximum</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr"/>
+      <c r="B10" s="3" t="inlineStr"/>
+      <c r="C10" s="3" t="inlineStr"/>
+      <c r="D10" s="3" t="inlineStr"/>
+      <c r="E10" s="3" t="inlineStr"/>
+      <c r="F10" s="3" t="inlineStr"/>
+      <c r="G10" s="3" t="inlineStr"/>
+      <c r="H10" s="3" t="inlineStr"/>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>Enter preferences and submit</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>System saves preferences and updates recommendation criteria</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>TC007</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>US32274</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Plan Personalization</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Negative - Invalid medication entry</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>User is authenticated</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>Medication: "" (blank entry)</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>Leave medication field blank and submit</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>System displays error: "Medication name required"</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>TC008</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>US32274</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Plan Personalization</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Edge - Large medication list</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>User is authenticated</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>Medication: 20+ entries</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>Enter 20+ medications and submit</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="inlineStr">
+        <is>
+          <t>System accepts all entries and processes recommendations without error</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>TC009</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>US32273</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Guided Enrollment</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Verify guided workflow for plan selection</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>User is a prospective member</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>Health: Asthma, PCP: Dr. Lee, Premium: $150</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>Start guided enrollment</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>System prompts for health data, provider, and financial preferences in sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr"/>
+      <c r="B14" s="3" t="inlineStr"/>
+      <c r="C14" s="3" t="inlineStr"/>
+      <c r="D14" s="3" t="inlineStr"/>
+      <c r="E14" s="3" t="inlineStr"/>
+      <c r="F14" s="3" t="inlineStr"/>
+      <c r="G14" s="3" t="inlineStr"/>
+      <c r="H14" s="3" t="inlineStr"/>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>Complete all steps and submit</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t>System generates and displays personalized plan recommendations with comparison tool</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>TC010</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>US32273</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Guided Enrollment</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Negative - Missing required fields</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>User is a prospective member</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>Omit required health data</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>Attempt to proceed without entering all required fields</t>
+        </is>
+      </c>
+      <c r="K15" s="3" t="inlineStr">
+        <is>
+          <t>System displays validation errors for missing fields</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>TC011</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>US32273</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Guided Enrollment</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Edge - Extreme cost preferences</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>User is a prospective member</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>Premium: $0, Deductible: $0</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>Enter extreme values and submit</t>
+        </is>
+      </c>
+      <c r="K16" s="3" t="inlineStr">
+        <is>
+          <t>System processes and displays only plans meeting criteria, or a message if none available</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>TC012</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>US31822</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Demographic Input</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Verify demographic and health needs input</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>User is a prospective member</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>Age: 40, Location: OH, Doctor: Dr. Adams, Medication: Lisinopril</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>Navigate to demographic input page</t>
+        </is>
+      </c>
+      <c r="K17" s="3" t="inlineStr">
+        <is>
+          <t>System displays fields for age, location, doctors, medications</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr"/>
+      <c r="B18" s="3" t="inlineStr"/>
+      <c r="C18" s="3" t="inlineStr"/>
+      <c r="D18" s="3" t="inlineStr"/>
+      <c r="E18" s="3" t="inlineStr"/>
+      <c r="F18" s="3" t="inlineStr"/>
+      <c r="G18" s="3" t="inlineStr"/>
+      <c r="H18" s="3" t="inlineStr"/>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>Enter data and submit</t>
+        </is>
+      </c>
+      <c r="K18" s="3" t="inlineStr">
+        <is>
+          <t>System validates and accepts input, proceeding to recommendations</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>TC013</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>US31822</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Demographic Input</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Negative - Invalid age</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>User is a prospective member</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>Age: -1</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>Enter invalid age and submit</t>
+        </is>
+      </c>
+      <c r="K19" s="3" t="inlineStr">
+        <is>
+          <t>System displays error: "Invalid age"</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>TC014</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>US31822</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Demographic Input</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Edge - Maximum field length</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>User is a prospective member</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>Doctor name: 100+ characters</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>Enter maximum length for doctor name and submit</t>
+        </is>
+      </c>
+      <c r="K20" s="3" t="inlineStr">
+        <is>
+          <t>System accepts or displays appropriate error without crashing</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>TC015</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>US32306</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Profile</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Verify profile view</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>User is logged in</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>User with profile data</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>Navigate to profile page</t>
+        </is>
+      </c>
+      <c r="K21" s="3" t="inlineStr">
+        <is>
+          <t>System displays correct profile information</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>TC016</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>US32307</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Settings</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Verify settings update</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>User is logged in</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>New notification preference</t>
+        </is>
+      </c>
+      <c r="I22" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>Go to settings, change preference, save</t>
+        </is>
+      </c>
+      <c r="K22" s="3" t="inlineStr">
+        <is>
+          <t>System updates and confirms setting change</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>TC017</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>US32308</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Transaction History</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>Verify transaction history view</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>User is logged in</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>User with transaction history</t>
+        </is>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J23" s="3" t="inlineStr">
+        <is>
+          <t>Navigate to transaction history</t>
+        </is>
+      </c>
+      <c r="K23" s="3" t="inlineStr">
+        <is>
+          <t>System displays all past transactions</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>TC018</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>US32309</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Search and Filter</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>Verify data search and filter</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>User is logged in</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>Search: "Diabetes", Filter: Date range</t>
+        </is>
+      </c>
+      <c r="I24" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J24" s="3" t="inlineStr">
+        <is>
+          <t>Enter search term and filter</t>
+        </is>
+      </c>
+      <c r="K24" s="3" t="inlineStr">
+        <is>
+          <t>System returns correct filtered data</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>TC019</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>US32310</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Export Reports</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>Verify report export</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>User is logged in</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>Report: Claims</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J25" s="3" t="inlineStr">
+        <is>
+          <t>Click export on claims report</t>
+        </is>
+      </c>
+      <c r="K25" s="3" t="inlineStr">
+        <is>
+          <t>System downloads report in selected format</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>TC020</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>US32311</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>User Permissions</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>Verify permission management</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>Admin user logged in</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>Assign 'Editor' to user X</t>
+        </is>
+      </c>
+      <c r="I26" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J26" s="3" t="inlineStr">
+        <is>
+          <t>Navigate to permissions, assign role</t>
+        </is>
+      </c>
+      <c r="K26" s="3" t="inlineStr">
+        <is>
+          <t>System saves and reflects new permission</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>TC021</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>US32312</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>System Logs</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>Verify system log view</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>Admin user logged in</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>Any log record</t>
+        </is>
+      </c>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J27" s="3" t="inlineStr">
+        <is>
+          <t>Navigate to system logs</t>
+        </is>
+      </c>
+      <c r="K27" s="3" t="inlineStr">
+        <is>
+          <t>System displays logs with timestamp, user, action</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>TC022</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>US32304</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Password Reset</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>Verify password reset</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>User on login page</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>Registered email</t>
+        </is>
+      </c>
+      <c r="I28" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J28" s="3" t="inlineStr">
+        <is>
+          <t>Click 'Forgot Password', enter email</t>
+        </is>
+      </c>
+      <c r="K28" s="3" t="inlineStr">
+        <is>
+          <t>System sends reset link to email</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>TC023</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>US32305</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Two-Factor Authentication</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>Verify 2FA enablement</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>User is logged in</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>Valid phone number</t>
+        </is>
+      </c>
+      <c r="I29" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J29" s="3" t="inlineStr">
+        <is>
+          <t>Navigate to security, enable 2FA</t>
+        </is>
+      </c>
+      <c r="K29" s="3" t="inlineStr">
+        <is>
+          <t>System sends code and confirms setup</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>TC024</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>US32303</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>Verify email login</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>User is registered</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>Valid email/password</t>
+        </is>
+      </c>
+      <c r="I30" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J30" s="3" t="inlineStr">
+        <is>
+          <t>Enter credentials, click login</t>
+        </is>
+      </c>
+      <c r="K30" s="3" t="inlineStr">
+        <is>
+          <t>System authenticates and redirects to dashboard</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>TC025</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>US32983</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>NEW STORY TETS</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>Basic smoke test</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>System available</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I31" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J31" s="3" t="inlineStr">
+        <is>
+          <t>Access feature</t>
+        </is>
+      </c>
+      <c r="K31" s="3" t="inlineStr">
+        <is>
+          <t>Feature loads without error</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>TC026</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>US32744</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>member 1</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>Basic smoke test</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>System available</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I32" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J32" s="3" t="inlineStr">
+        <is>
+          <t>Access feature</t>
+        </is>
+      </c>
+      <c r="K32" s="3" t="inlineStr">
+        <is>
+          <t>Feature loads without error</t>
         </is>
       </c>
     </row>

</xml_diff>